<commit_message>
feat: :tada: Add new project
Change the word to pdf, and add .env in this project
</commit_message>
<xml_diff>
--- a/registro_chat.xlsx
+++ b/registro_chat.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,6 +488,35 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Un adolescente fue retenido por la policía sin orden judicial mientras caminaba por la calle, sin cometer delito aparente. ¿Es legal esta retención según el Código de la Niñez y Adolescencia?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>El contexto legal proporcionado no ofrece información sobre la legalidad de la detención de un adolescente sin orden judicial mientras camina por la calle sin cometer un delito aparente.  Los artículos 351, 256, 261 y 262 del Código de la Niñez y Adolescencia, citados,  se refieren respectivamente a la remisión con autorización judicial, los principios rectores de la administración de justicia especializada en niñez y adolescencia,  normas supletorias y la competencia de los jueces de adolescentes infractores.  Ninguno de estos artículos aborda la cuestión de la detención arbitraria de un menor sin orden judicial.  Por lo tanto, basándome únicamente en el texto legal proporcionado, no puedo determinar la legalidad de la acción policial descrita.  Se requiere información adicional sobre las leyes que regulan las detenciones de menores para emitir un juicio.
+Veredicto final:  No hay información suficiente en el contexto legal proporcionado para determinar la legalidad de la retención del adolescente. Se necesita información legal adicional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Un adolescente de 16 años trabaja seis días a la semana durante ocho horas diarias en una fábrica. Su jornada laboral no le permite asistir regularmente a clases. ¿Este tipo de trabajo vulnera los derechos establecidos en el Código de la Niñez y Adolescencia? ¿Qué disposiciones legales se aplican y cuál sería el veredicto correspondiente?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>El caso presentado involucra a un adolescente de 16 años que trabaja seis días a la semana, ocho horas diarias en una fábrica, imposibilitándole asistir regularmente a clases.  Debemos determinar si esta situación vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, basándonos únicamente en el texto legal proporcionado.
+El artículo 91 del Código de la Niñez y Adolescencia, aunque se refiere al trabajo doméstico, establece que los adolescentes trabajadores tienen derechos y garantías generales.  Si bien no detalla específicamente las horas máximas de trabajo, el contexto legal implica la protección del adolescente contra la explotación laboral. El artículo 89, aunque no se cita explícitamente en el contexto, se infiere su aplicación por la referencia a la protección contra la explotación laboral, y éste debe ser interpretado en conjunto con el resto de normas. El artículo 89 del Código de la Niñez y Adolescencia declara el derecho de los niños, niñas y adolescentes a la protección contra la explotación laboral, incluyendo cualquier trabajo nocivo para su salud, desarrollo o que entorpezca su derecho a la educación.  La jornada laboral descrita, de seis días a la semana por ocho horas diarias, impide la asistencia regular a clases, lo cual constituye una clara vulneración del derecho a la educación y, por ende, una forma de explotación laboral según la interpretación del Art. 89.
+Además, el texto legal menciona la obligación del patrono de registrar el contrato de trabajo (aunque no especifica sanciones por incumplimiento). La ausencia de registro, en este caso, es un factor adicional que contribuye a la vulneración de los derechos del adolescente.  La falta de un contrato escrito no exime al empleador de su responsabilidad.
+Considerando la extenuante jornada laboral que impide la asistencia regular a la escuela y la posibilidad implícita del incumplimiento de registro del contrato, concluyo que la situación descrita infringe los derechos del adolescente establecidos en el Código de la Niñez y Adolescencia, especialmente el derecho a la protección contra la explotación laboral y el derecho a la educación,  deducible del Art. 89 y consistente con el espíritu del Art. 91.
+Veredicto final: Se declara que el trabajo realizado por el adolescente de 16 años vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, específicamente su derecho a la educación y a la protección contra la explotación laboral.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: :hammer: Update file
add new row in excel for time the question
</commit_message>
<xml_diff>
--- a/registro_chat.xlsx
+++ b/registro_chat.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,93 +427,94 @@
           <t>Respuesta</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tiempo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>¿Cuales son tus horarios?</t>
+          <t>Un padre castiga a su hijo de 11 años con bofetadas frecuentes y amenazas verbales. El niño muestra signos de afectación emocional y retraimiento. ¿Esta conducta constituye maltrato bajo la normativa vigente sobre niñez y adolescencia en Ecuador? ¿Qué medidas podrían adoptarse legalmente frente a esta situación?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Los horarios de atención de la matriz en Carapungo son de lunes a jueves de 8 am a 8 pm, viernes de 8 am a 6 pm, sábados solo para emergencias y domingos de 7:30 am a 7:30 pm.  La sucursal de Llano Grande atiende de lunes a jueves de 7 am a 10 pm, viernes de 7 am a 6 pm, sábados no hay atención y domingos de 7 am a 10 pm.  En feriados se atiende con normalidad, excepto los sábados.</t>
+          <t>El caso presentado describe una situación donde un padre castiga a su hijo de 11 años con bofetadas frecuentes y amenazas verbales, causando afectación emocional y retraimiento en el menor.  El contexto legal proporcionado, aunque incompleto, alude a la protección de los niños, niñas y adolescentes frente al maltrato.  Si bien no se proporciona un artículo específico que defina explícitamente "bofetadas frecuentes y amenazas verbales" como maltrato,  el fragmento del artículo 7 referente a "hogares cuyos miembros tengan antecedentes como autores de abuso o maltrato" permite inferir que este tipo de acciones son susceptibles de ser consideradas como tal.  El hecho de que el niño presente signos de afectación emocional y retraimiento corrobora la presencia de daño, lo cual se alinea con el espíritu protector de los artículos sobre los derechos de la niñez,  como el derecho a la recreación, al descanso y el desarrollo integral (Art. 48, aunque incompleto en el contexto).  Adicionalmente, el Art. 269, que trata sobre la investigación para ubicar a padres ausentes o desaparecidos, aunque no se aplica directamente al caso presente, refuerza la obligación del Estado de proteger a los niños, niñas y adolescentes.  
+La ausencia de definiciones precisas en el contexto legal proporcionado dificulta una calificación definitiva de la conducta del padre bajo una tipificación específica de maltrato. Sin embargo, la evidencia de daño emocional al menor, conjuntamente con las acciones descritas (bofetadas y amenazas), permiten concluir que existe una alta probabilidad de que la conducta del padre constituya una forma de maltrato infantil, violentando el espíritu protector de la legislación ecuatoriana sobre niñez y adolescencia.
+En consecuencia, ante la posibilidad de que se esté infringiendo la protección legal del niño, se debería proceder a una investigación exhaustiva para determinar si la conducta del padre se ajusta a una figura legal de maltrato infantil.  De confirmarse, se podrían adoptar las medidas legales pertinentes para proteger al menor, las cuales podrían incluir, pero no se limitan a, medidas de protección del niño,  intervención con el padre para modificar su conducta, o incluso, si el nivel de afectación al menor lo requiere, la separación del menor del padre. La decisión final sobre las medidas a adoptar dependerá de una investigación completa, realizada por la autoridad competente y teniendo en cuenta el contexto completo de la legislación ecuatoriana sobre niñez y adolescencia, más allá del fragmento proporcionado.
+Veredicto final: Dada la información suministrada,  se concluye que existe la fuerte sospecha de maltrato infantil. Se ordena una investigación a fondo para determinar la existencia de maltrato según la legislación ecuatoriana sobre niñez y adolescencia y para aplicar las medidas de protección al menor que sean necesarias.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>atienden en feriado</t>
+          <t>Un adolescente de 16 años trabaja seis días a la semana durante ocho horas diarias en una fábrica. Su jornada laboral no le permite asistir regularmente a clases. ¿Este tipo de trabajo vulnera los derechos establecidos en el Código de la Niñez y Adolescencia? ¿Qué disposiciones legales se aplican y cuál sería el veredicto correspondiente?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sí, atienden en todos los feriados con normalidad, excepto los sábados.</t>
+          <t>El caso presentado involucra a un adolescente de 16 años que trabaja seis días a la semana, ocho horas diarias en una fábrica, imposibilitándole la asistencia regular a clases.  Debemos determinar si esta situación vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, basándonos únicamente en el contexto legal proporcionado.
+El artículo referente al derecho a la protección contra la explotación laboral,  establece que los niños, niñas y adolescentes tienen derecho a la protección contra la explotación laboral y económica, y cualquier forma de trabajo nocivo para su salud, desarrollo físico, mental, espiritual, moral o social, o que pueda entorpecer el ejercicio de su derecho a la educación.  La situación descrita, donde un adolescente de 16 años trabaja seis días a la semana, ocho horas diarias,  claramente impide el ejercicio regular de su derecho a la educación.  Este trabajo, por su intensidad horaria y su interferencia directa con su educación, puede ser considerado  "nocivo para su desarrollo" y  "que puede entorpecer el ejercicio de su derecho a la educación", tal como lo define el artículo mencionado.
+Adicionalmente, aunque el contexto legal no especifica un límite de horas para el trabajo de un adolescente de 16 años, la imposibilidad de asistir regularmente a clases por causa del trabajo sugiere una clara vulneración de sus derechos. La legislación resalta la prioridad de las exigencias pedagógicas sobre los objetivos productivos en cualquier programa que incorpore trabajo adolescente.  El trabajo descrito claramente prioriza el objetivo productivo sobre el desarrollo integral del adolescente, incumpliendo este principio implícito en el texto legal.
+El hecho de que el adolescente trabaje en una fábrica, sin más detalles, no permite determinar si se cumple con el registro del contrato de trabajo según lo establecido en la legislación.  Sin embargo,  la violación al derecho a la educación, en sí misma, es suficiente para determinar la vulneración de derechos.
+Por lo tanto, considerando el contexto legal proporcionado, se concluye que el trabajo del adolescente de 16 años, bajo las condiciones descritas, vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, específicamente su derecho a la protección contra la explotación laboral y su derecho a la educación.
+Veredicto final: Se declara que el trabajo del adolescente de 16 años en la fábrica, con una jornada de seis días a la semana y ocho horas diarias, vulnera sus derechos, según el Código de la Niñez y Adolescencia.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>40</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>hay vacunas</t>
+          <t>Un adolescente de 16 años trabaja ocho horas diarias en un taller mecánico, seis días a la semana. Esta jornada le impide asistir regularmente al colegio. Según el Código de la Niñez y Adolescencia, especialmente en lo dispuesto sobre jornada laboral, derecho a la educación y trabajo prohibido para adolescentes, ¿esta situación vulnera sus derechos? ¿Qué artículos serían aplicables y qué medidas deberían tomarse?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sí, hay vacunas para perros y gatos.  Para perros se ofrecen vacunas Puppy, Rabia, Bordetella y Múltiple. Para gatos, las vacunas disponibles son Triple Felina, Leucemia Felina y Rabia. El número de vacunas para perros depende de la edad en que se inicia el plan vacunal. Las vacunas anuales para perros (Múltiple, Bordetella, Rabia) tienen un costo de $15 cada una e incluyen desparasitación.</t>
+          <t>El caso presentado se centra en un adolescente de 16 años que trabaja ocho horas diarias, seis días a la semana en un taller mecánico, situación que le impide asistir regularmente al colegio.  Debemos determinar si esta situación vulnera sus derechos conforme al Código de la Niñez y Adolescencia.
+El artículo que regula directamente el trabajo de adolescentes es el artículo 91, que establece que los adolescentes que trabajan en servicio doméstico tienen los mismos derechos y garantías que los adolescentes trabajadores en general.  Aunque el caso no se refiere a trabajo doméstico, el principio de igualdad de derechos para adolescentes trabajadores se extiende implícitamente a otros tipos de trabajo.  El artículo además establece que el patrono debe velar por la integridad física, psicológica y moral del adolescente y garantizar sus derechos a la alimentación y educación.  La jornada laboral de ocho horas diarias, seis días a la semana, claramente impide el ejercicio del derecho a la educación del adolescente, vulnerando lo dispuesto en este artículo.
+Adicionalmente, el derecho a la protección contra la explotación laboral, implícito en el Código de la Niñez y Adolescencia y concordante con artículos del Código del Trabajo (no proporcionados en su totalidad en el contexto), se ve vulnerado.  La jornada laboral extensa y la imposibilidad de asistir al colegio constituyen explotación laboral, ya que perjudican su desarrollo físico, mental y su derecho a la educación.
+El artículo 374 establece la competencia de los juzgadores especializados en adolescentes infractores para el control jurisdiccional de las medidas socioeducativas.  Si bien este artículo no dictamina directamente sobre la presente situación, sienta la base para la aplicación de medidas correctivas, si se determina una infracción.  El contexto legal no ofrece información sobre las sanciones específicas para este tipo de violación de derechos.  Sin embargo, la gravedad de la situación, la explotación laboral manifiesta y la violación al derecho a la educación ameritan la intervención de las autoridades competentes para proteger al menor.
+En conclusión, la situación descrita vulnera los derechos del adolescente de 16 años, infringiendo los principios de protección contra la explotación laboral y el derecho a la educación, conforme a la interpretación del artículo 91 del Código de la Niñez y Adolescencia y los principios concordantes con el Código del Trabajo.  Se requiere la intervención de los juzgadores especializados en adolescentes infractores para determinar las medidas correctivas pertinentes, conforme al artículo 374 del mismo código,  para garantizar la protección del menor y el cumplimiento de sus derechos.
+Veredicto final: Se declara la vulneración de los derechos del adolescente de 16 años y se ordena la intervención de los juzgadores especializados en adolescentes infractores para determinar las medidas socioeducativas apropiadas para remediar la situación, en concordancia con el artículo 374 del Código de la Niñez y Adolescencia y los principios concordantes con el Código del Trabajo.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>54</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tuve una infraccion por mi auto mal estacionacionado</t>
+          <t>Una niña recién nacida no fue inscrita en el Registro Civil dentro de las semanas posteriores a su nacimiento debido a la negligencia del centro de salud y la falta de información proporcionada a la madre. Conforme a la normativa del Código de la Niñez y Adolescencia, ¿qué derechos de la niña han sido vulnerados y qué responsabilidades tienen tanto el establecimiento de salud como el Estado en esta situación?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>El texto proporcionado no contiene información sobre infracciones de estacionamiento.  Por lo tanto, no puedo responder a tu pregunta usando solo la información dada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tuve una infraccion por mi auto mal estacionacionado</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Lo siento, pero no puedo ayudarte con tu infracción de estacionamiento. El texto proporcionado solo contiene "BIENVINDOS A L T C", que no proporciona información relevante sobre multas de tráfico o estacionamiento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Un adolescente fue retenido por la policía sin orden judicial mientras caminaba por la calle, sin cometer delito aparente. ¿Es legal esta retención según el Código de la Niñez y Adolescencia?</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>El contexto legal proporcionado no ofrece información sobre la legalidad de la detención de un adolescente sin orden judicial mientras camina por la calle sin cometer un delito aparente.  Los artículos 351, 256, 261 y 262 del Código de la Niñez y Adolescencia, citados,  se refieren respectivamente a la remisión con autorización judicial, los principios rectores de la administración de justicia especializada en niñez y adolescencia,  normas supletorias y la competencia de los jueces de adolescentes infractores.  Ninguno de estos artículos aborda la cuestión de la detención arbitraria de un menor sin orden judicial.  Por lo tanto, basándome únicamente en el texto legal proporcionado, no puedo determinar la legalidad de la acción policial descrita.  Se requiere información adicional sobre las leyes que regulan las detenciones de menores para emitir un juicio.
-Veredicto final:  No hay información suficiente en el contexto legal proporcionado para determinar la legalidad de la retención del adolescente. Se necesita información legal adicional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Un adolescente de 16 años trabaja seis días a la semana durante ocho horas diarias en una fábrica. Su jornada laboral no le permite asistir regularmente a clases. ¿Este tipo de trabajo vulnera los derechos establecidos en el Código de la Niñez y Adolescencia? ¿Qué disposiciones legales se aplican y cuál sería el veredicto correspondiente?</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>El caso presentado involucra a un adolescente de 16 años que trabaja seis días a la semana, ocho horas diarias en una fábrica, imposibilitándole asistir regularmente a clases.  Debemos determinar si esta situación vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, basándonos únicamente en el texto legal proporcionado.
-El artículo 91 del Código de la Niñez y Adolescencia, aunque se refiere al trabajo doméstico, establece que los adolescentes trabajadores tienen derechos y garantías generales.  Si bien no detalla específicamente las horas máximas de trabajo, el contexto legal implica la protección del adolescente contra la explotación laboral. El artículo 89, aunque no se cita explícitamente en el contexto, se infiere su aplicación por la referencia a la protección contra la explotación laboral, y éste debe ser interpretado en conjunto con el resto de normas. El artículo 89 del Código de la Niñez y Adolescencia declara el derecho de los niños, niñas y adolescentes a la protección contra la explotación laboral, incluyendo cualquier trabajo nocivo para su salud, desarrollo o que entorpezca su derecho a la educación.  La jornada laboral descrita, de seis días a la semana por ocho horas diarias, impide la asistencia regular a clases, lo cual constituye una clara vulneración del derecho a la educación y, por ende, una forma de explotación laboral según la interpretación del Art. 89.
-Además, el texto legal menciona la obligación del patrono de registrar el contrato de trabajo (aunque no especifica sanciones por incumplimiento). La ausencia de registro, en este caso, es un factor adicional que contribuye a la vulneración de los derechos del adolescente.  La falta de un contrato escrito no exime al empleador de su responsabilidad.
-Considerando la extenuante jornada laboral que impide la asistencia regular a la escuela y la posibilidad implícita del incumplimiento de registro del contrato, concluyo que la situación descrita infringe los derechos del adolescente establecidos en el Código de la Niñez y Adolescencia, especialmente el derecho a la protección contra la explotación laboral y el derecho a la educación,  deducible del Art. 89 y consistente con el espíritu del Art. 91.
-Veredicto final: Se declara que el trabajo realizado por el adolescente de 16 años vulnera los derechos establecidos en el Código de la Niñez y Adolescencia, específicamente su derecho a la educación y a la protección contra la explotación laboral.</t>
+          <t>El caso presentado describe la vulneración del derecho a la identidad de la niña recién nacida, amparado en el Código de la Niñez y Adolescencia.  Si bien el contexto legal no especifica un plazo explícito para la inscripción en el Registro Civil, la omisión del centro de salud en realizarla y la falta de información a la madre constituyen una negligencia que impide el ejercicio pleno del derecho a la identidad, garantizado implícitamente por el derecho a la salud (acceso a los programas y acciones de salud públicos) y el derecho a la protección integral que el Estado debe garantizar según el artículo 1. La falta de inscripción impide el acceso a otros derechos, como el acceso a servicios de salud y educación.
+El artículo 1 del Código de la Niñez y Adolescencia establece la finalidad de protección integral que el Estado debe garantizar a los niños, niñas y adolescentes.  Esta protección integral incluye, necesariamente, la efectiva inscripción en el Registro Civil, acto fundamental para el ejercicio de la ciudadanía y el acceso a los servicios básicos.  La falta de inscripción, causada por la negligencia del centro de salud, representa una violación directa de esta obligación estatal de protección.
+Además, el artículo referente a las obligaciones de los establecimientos de salud, aunque no menciona explícitamente la inscripción en el Registro Civil,  establece la obligación de prestar servicios, incluyendo implícitamente la información y orientación necesaria para el pleno ejercicio de los derechos del niño, niña o adolescente.  La omisión en brindar esta información sobre la inscripción, constituye una negligencia que configura una violación de la obligación establecida en dicho artículo.
+Por tanto, la responsabilidad del establecimiento de salud radica en su negligencia al no realizar la inscripción y al no informar adecuadamente a la madre. La responsabilidad del Estado reside en la falta de supervisión y control  sobre el cumplimiento de las obligaciones de los centros de salud en cuanto a la garantía de los derechos de los niños, niñas y adolescentes.  El Estado, a través de sus instituciones, tiene la obligación de velar por el cumplimiento de las normas del Código de la Niñez y Adolescencia.
+Veredicto final: Se declara la vulneración de los derechos de la niña recién nacida, específicamente su derecho a la identidad. Se determina la responsabilidad del establecimiento de salud por negligencia en la inscripción y falta de información a la madre, y la responsabilidad del Estado por falta de supervisión y garantía del cumplimiento de las obligaciones de los centros de salud. Se ordena al establecimiento de salud realizar la inscripción de la niña en el Registro Civil de manera inmediata y se recomienda a las autoridades competentes implementar medidas para prevenir situaciones similares en el futuro.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>38</t>
         </is>
       </c>
     </row>

</xml_diff>